<commit_message>
dynamic allocation and teacher dashboard fixed
</commit_message>
<xml_diff>
--- a/uploads/class_type.xlsx
+++ b/uploads/class_type.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\float_working2\data\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482E63BB-337B-47C4-B1DE-E088B1AA6D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A770B630-E0AE-4142-9C10-2ACC9423773D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="144">
   <si>
     <t>subject</t>
   </si>
@@ -428,13 +428,37 @@
   </si>
   <si>
     <t>Project</t>
+  </si>
+  <si>
+    <t>W/S EE/W/S EC</t>
+  </si>
+  <si>
+    <t>CHEM LAB/W/S EE</t>
+  </si>
+  <si>
+    <t>CHEM LAB/W/S EC</t>
+  </si>
+  <si>
+    <t>CED LAB</t>
+  </si>
+  <si>
+    <t>CHEMISTRY LAB/IT W/S</t>
+  </si>
+  <si>
+    <t>PC LAB Lab/IT W/S</t>
+  </si>
+  <si>
+    <t>Chem lab/ IT Lab</t>
+  </si>
+  <si>
+    <t>OS LAB/DBMS LAB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -456,6 +480,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -493,7 +523,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -502,6 +532,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,7 +837,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B137"/>
+  <dimension ref="A1:B145"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38.33203125" customWidth="1"/>
@@ -1909,7 +1940,72 @@
         <v>12</v>
       </c>
     </row>
+    <row r="138" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A138" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B138" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>137</v>
+      </c>
+      <c r="B139" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>138</v>
+      </c>
+      <c r="B140" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>139</v>
+      </c>
+      <c r="B141" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>140</v>
+      </c>
+      <c r="B142" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>141</v>
+      </c>
+      <c r="B143" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>142</v>
+      </c>
+      <c r="B144" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>143</v>
+      </c>
+      <c r="B145" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>